<commit_message>
update raw data file
</commit_message>
<xml_diff>
--- a/data-raw/rawdata_edited.xlsx
+++ b/data-raw/rawdata_edited.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawkels\Kelsey - Caetano - Linda\Sampling &amp; Field &amp; Lab\Raw Data\0 - raw_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawkels\Kelsey - Caetano - Linda\5_Data\01_field_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D9FD2E-CF55-46A2-ABC9-188AF558752A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="661"/>
+    <workbookView xWindow="12800" yWindow="0" windowWidth="12800" windowHeight="13800" tabRatio="661" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="16" r:id="rId1"/>
@@ -17,7 +18,7 @@
     <sheet name="gas" sheetId="28" r:id="rId3"/>
     <sheet name="parameters" sheetId="15" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1015,7 +1016,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
@@ -1147,7 +1148,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="fmtMidLeft" xfId="1"/>
+    <cellStyle name="fmtMidLeft" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1465,7 +1466,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AM42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -6103,7 +6104,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -7472,8 +7473,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G111"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:J111"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.6328125" bestFit="1" customWidth="1"/>
@@ -7484,7 +7485,7 @@
     <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>132</v>
       </c>
@@ -7506,8 +7507,10 @@
       <c r="G1" s="4" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>7</v>
       </c>
@@ -7521,7 +7524,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="5">
-        <v>2.636158905904523</v>
+        <v>27.256032960311835</v>
       </c>
       <c r="F2" s="10">
         <v>0</v>
@@ -7529,8 +7532,10 @@
       <c r="G2" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -7544,16 +7549,18 @@
         <v>3</v>
       </c>
       <c r="E3" s="5">
-        <v>0.60373304087214053</v>
+        <v>31.683908747629939</v>
       </c>
       <c r="F3" s="10">
-        <v>0</v>
+        <v>87.434598130127654</v>
       </c>
       <c r="G3" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
@@ -7567,16 +7574,18 @@
         <v>2</v>
       </c>
       <c r="E4" s="5">
-        <v>1.6219944898894096</v>
+        <v>7.0569646960259611</v>
       </c>
       <c r="F4" s="10">
-        <v>0</v>
+        <v>63.143274473722634</v>
       </c>
       <c r="G4" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
@@ -7590,16 +7599,18 @@
         <v>3</v>
       </c>
       <c r="E5" s="5">
-        <v>1.3010745781164941</v>
+        <v>40.083047620107997</v>
       </c>
       <c r="F5" s="10">
-        <v>0</v>
+        <v>19.32545041520487</v>
       </c>
       <c r="G5" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>14</v>
       </c>
@@ -7613,16 +7624,16 @@
         <v>2</v>
       </c>
       <c r="E6" s="5">
-        <v>6.2442928261726101</v>
+        <v>85.619676672652588</v>
       </c>
       <c r="F6" s="10">
-        <v>49.42965571262723</v>
+        <v>161.51600270489382</v>
       </c>
       <c r="G6" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -7637,7 +7648,7 @@
         <v>410</v>
       </c>
       <c r="E7" s="5">
-        <v>6.9874856720334708E-2</v>
+        <v>0.41804215414344859</v>
       </c>
       <c r="F7" s="10">
         <v>0</v>
@@ -7646,7 +7657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -7660,7 +7671,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="5">
-        <v>1.7547574474127787</v>
+        <v>41.581268461004157</v>
       </c>
       <c r="F8" s="10">
         <v>0</v>
@@ -7669,7 +7680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
@@ -7683,16 +7694,16 @@
         <v>2</v>
       </c>
       <c r="E9" s="5">
-        <v>6.9684218922271048</v>
+        <v>116.9319533376742</v>
       </c>
       <c r="F9" s="10">
-        <v>0</v>
+        <v>179.60486212833976</v>
       </c>
       <c r="G9" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
@@ -7715,7 +7726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
@@ -7729,16 +7740,16 @@
         <v>368</v>
       </c>
       <c r="E11" s="5">
-        <v>6.3242229995352298E-2</v>
+        <v>1.1288055659963265</v>
       </c>
       <c r="F11" s="10">
-        <v>0</v>
+        <v>0.39877288001502859</v>
       </c>
       <c r="G11" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -7752,16 +7763,16 @@
         <v>4</v>
       </c>
       <c r="E12" s="5">
-        <v>3.7113810141010423E-2</v>
+        <v>0.16777941727158485</v>
       </c>
       <c r="F12" s="10">
-        <v>0</v>
+        <v>3.4966994406334519</v>
       </c>
       <c r="G12" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -7775,16 +7786,16 @@
         <v>2</v>
       </c>
       <c r="E13" s="5">
-        <v>3.0477408485254385</v>
+        <v>14.571948977041183</v>
       </c>
       <c r="F13" s="10">
-        <v>2.203290852651111</v>
+        <v>19.803629333789317</v>
       </c>
       <c r="G13" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -7798,7 +7809,7 @@
         <v>10</v>
       </c>
       <c r="E14" s="5">
-        <v>3.8736863075649837E-2</v>
+        <v>3.4719943236557458</v>
       </c>
       <c r="F14" s="10">
         <v>0</v>
@@ -7807,7 +7818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
@@ -7821,16 +7832,16 @@
         <v>2</v>
       </c>
       <c r="E15" s="5">
-        <v>14.241294116190522</v>
+        <v>153.2423560757739</v>
       </c>
       <c r="F15" s="10">
-        <v>0</v>
+        <v>176.11862559465976</v>
       </c>
       <c r="G15" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>35</v>
       </c>
@@ -7867,10 +7878,10 @@
         <v>3</v>
       </c>
       <c r="E17" s="5">
-        <v>3.6979108812784931</v>
+        <v>28.485341453873755</v>
       </c>
       <c r="F17" s="10">
-        <v>15.913642332138245</v>
+        <v>81.11974136168314</v>
       </c>
       <c r="G17" s="2">
         <v>0</v>
@@ -7890,7 +7901,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="5">
-        <v>4.5469290015537265</v>
+        <v>30.760164271592441</v>
       </c>
       <c r="F18" s="10">
         <v>0</v>
@@ -7913,7 +7924,7 @@
         <v>2</v>
       </c>
       <c r="E19" s="5">
-        <v>10.370416059605184</v>
+        <v>15.209500495155361</v>
       </c>
       <c r="F19" s="10">
         <v>0</v>
@@ -7936,10 +7947,10 @@
         <v>3</v>
       </c>
       <c r="E20" s="5">
-        <v>0.97299809427969042</v>
+        <v>36.117419601049299</v>
       </c>
       <c r="F20" s="10">
-        <v>6.8247044192230932</v>
+        <v>59.718406767352484</v>
       </c>
       <c r="G20" s="2">
         <v>0</v>
@@ -7959,7 +7970,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="5">
-        <v>1.9281240383078269</v>
+        <v>13.691699720391201</v>
       </c>
       <c r="F21" s="10">
         <v>0</v>
@@ -7982,10 +7993,10 @@
         <v>200</v>
       </c>
       <c r="E22" s="5">
-        <v>0.16598108903827372</v>
+        <v>0.78425223654444509</v>
       </c>
       <c r="F22" s="10">
-        <v>0</v>
+        <v>1.3278801150469495</v>
       </c>
       <c r="G22" s="2">
         <v>0</v>
@@ -8028,10 +8039,10 @@
         <v>23</v>
       </c>
       <c r="E24" s="5">
-        <v>4.46</v>
+        <v>40.760529746994699</v>
       </c>
       <c r="F24" s="10">
-        <v>0</v>
+        <v>77.837928292732087</v>
       </c>
       <c r="G24" s="2">
         <v>0</v>
@@ -8051,10 +8062,10 @@
         <v>4</v>
       </c>
       <c r="E25" s="5">
-        <v>2.15</v>
+        <v>13.78189684420064</v>
       </c>
       <c r="F25" s="10">
-        <v>0</v>
+        <v>489.5511674618088</v>
       </c>
       <c r="G25" s="2">
         <v>0</v>
@@ -8073,11 +8084,11 @@
       <c r="D26" s="14">
         <v>5</v>
       </c>
-      <c r="E26" s="5">
-        <v>4.28</v>
+      <c r="E26">
+        <v>13.922565398619984</v>
       </c>
       <c r="F26" s="10">
-        <v>0</v>
+        <v>142.94185913569089</v>
       </c>
       <c r="G26" s="2">
         <v>0</v>
@@ -8097,7 +8108,7 @@
         <v>4</v>
       </c>
       <c r="E27" s="5">
-        <v>10.96</v>
+        <v>37.863042537419226</v>
       </c>
       <c r="F27" s="10">
         <v>0</v>
@@ -8120,7 +8131,7 @@
         <v>15</v>
       </c>
       <c r="E28" s="5">
-        <v>4.6900000000000004</v>
+        <v>21.609484786801232</v>
       </c>
       <c r="F28" s="10">
         <v>0</v>
@@ -8143,10 +8154,10 @@
         <v>9</v>
       </c>
       <c r="E29" s="5">
-        <v>2.1</v>
+        <v>16.940467516231084</v>
       </c>
       <c r="F29" s="10">
-        <v>0</v>
+        <v>16.250904483447439</v>
       </c>
       <c r="G29" s="2">
         <v>0</v>
@@ -8166,10 +8177,10 @@
         <v>15</v>
       </c>
       <c r="E30" s="5">
-        <v>1.87</v>
+        <v>6.9014015313100829</v>
       </c>
       <c r="F30" s="10">
-        <v>0</v>
+        <v>23.360308160919679</v>
       </c>
       <c r="G30" s="2">
         <v>0</v>
@@ -8189,7 +8200,7 @@
         <v>14</v>
       </c>
       <c r="E31" s="5">
-        <v>0.46</v>
+        <v>0.68228053039211889</v>
       </c>
       <c r="F31" s="10">
         <v>0</v>
@@ -8212,10 +8223,10 @@
         <v>35</v>
       </c>
       <c r="E32" s="5">
-        <v>0.2</v>
+        <v>0.76502851822708029</v>
       </c>
       <c r="F32" s="10">
-        <v>0</v>
+        <v>7.739177459094555</v>
       </c>
       <c r="G32" s="2">
         <v>0</v>
@@ -8235,10 +8246,10 @@
         <v>30</v>
       </c>
       <c r="E33" s="5">
-        <v>3.4</v>
+        <v>18.99466229724479</v>
       </c>
       <c r="F33" s="10">
-        <v>32.200000000000003</v>
+        <v>160.38552456591518</v>
       </c>
       <c r="G33" s="2">
         <v>0</v>
@@ -8258,10 +8269,10 @@
         <v>30</v>
       </c>
       <c r="E34" s="5">
-        <v>1.19</v>
+        <v>10.905486816804119</v>
       </c>
       <c r="F34" s="10">
-        <v>1.1000000000000001</v>
+        <v>31.764058108059167</v>
       </c>
       <c r="G34" s="2">
         <v>0</v>
@@ -8281,10 +8292,10 @@
         <v>88</v>
       </c>
       <c r="E35" s="5">
-        <v>7.98</v>
+        <v>25.183914185723339</v>
       </c>
       <c r="F35" s="10">
-        <v>0.9</v>
+        <v>39.861061346201026</v>
       </c>
       <c r="G35" s="2">
         <v>0</v>
@@ -8304,10 +8315,10 @@
         <v>35</v>
       </c>
       <c r="E36" s="5">
-        <v>1.44</v>
+        <v>12.560183791534289</v>
       </c>
       <c r="F36" s="10">
-        <v>0</v>
+        <v>33.035650424532093</v>
       </c>
       <c r="G36" s="2">
         <v>0</v>
@@ -8327,10 +8338,10 @@
         <v>43</v>
       </c>
       <c r="E37" s="5">
-        <v>0.9</v>
+        <v>3.2521696824356239</v>
       </c>
       <c r="F37" s="10">
-        <v>0</v>
+        <v>15.046435130031679</v>
       </c>
       <c r="G37" s="2">
         <v>0</v>
@@ -8350,10 +8361,10 @@
         <v>29</v>
       </c>
       <c r="E38" s="5">
-        <v>1.45</v>
+        <v>5.2923871983452093</v>
       </c>
       <c r="F38" s="10">
-        <v>1</v>
+        <v>9.689658198069047</v>
       </c>
       <c r="G38" s="2">
         <v>0</v>
@@ -8376,7 +8387,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="10">
-        <v>1.6</v>
+        <v>19.447947290655982</v>
       </c>
       <c r="G39" s="2">
         <v>0</v>
@@ -8396,10 +8407,10 @@
         <v>16</v>
       </c>
       <c r="E40" s="5">
-        <v>3.04</v>
+        <v>41.48733670085722</v>
       </c>
       <c r="F40" s="10">
-        <v>1.8</v>
+        <v>71.687198413046801</v>
       </c>
       <c r="G40" s="2">
         <v>0</v>
@@ -8419,10 +8430,10 @@
         <v>52</v>
       </c>
       <c r="E41" s="5">
-        <v>1.41</v>
+        <v>4.6043646132977205</v>
       </c>
       <c r="F41" s="10">
-        <v>1.1000000000000001</v>
+        <v>8.8582875515555664</v>
       </c>
       <c r="G41" s="2">
         <v>0</v>
@@ -8442,10 +8453,10 @@
         <v>14</v>
       </c>
       <c r="E42" s="5">
-        <v>0.49</v>
+        <v>3.5666395482277267</v>
       </c>
       <c r="F42" s="10">
-        <v>0</v>
+        <v>25.965908032387219</v>
       </c>
       <c r="G42" s="2">
         <v>0</v>
@@ -9079,7 +9090,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AC122"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>